<commit_message>
feat(infra): scaffold single-environment Terraform on Hetzner (US-003)
Single CX23 (fsn1) running app, PDF worker, Postgres and Redis
co-located, as a temporary pre-launch descope from the three
isolated environments US-003 originally called for. Remote state
in Hetzner Object Storage (S3-compatible). infra/README.md and
the backlog's US-003 acceptance criteria updated to document the
descope and what must land before real users or payments go live.

Also carries the earlier US-001 status update in the same backlog
file (uncommitted until now).
</commit_message>
<xml_diff>
--- a/docs/planning/Jyotish_DE_Backlog_v3.xlsx
+++ b/docs/planning/Jyotish_DE_Backlog_v3.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Launch Checklist" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors &amp; Costs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team &amp; Effort" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Epics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="User Stories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Release Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tech Launch Checklist" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Vendors &amp; Costs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Team &amp; Effort" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'User Stories'!$A$1:$M$114</definedName>
@@ -645,9 +645,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2103,7 +2100,7 @@
       <c r="K2" s="7" t="inlineStr"/>
       <c r="L2" s="9" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr"/>
@@ -2197,7 +2194,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>1) All compute, DB, storage and backups in eu-central-1 (Frankfurt). 2) No production data in dev or staging. 3) Secrets in a managed store, never in the repo. 4) Defined in IaC and reproducible.</t>
+          <t>1) All compute, DB, storage and backups in eu-central-1 (Frankfurt). 2) No production data in dev or staging. 3) Secrets in a managed store, never in the repo. 4) Defined in IaC and reproducible. DESCOPED (2026-08-01): single environment only for now (Hetzner, fsn1), pre-launch/pre-real-users — see infra/README.md. Full dev/staging/prod split must land before real users or payments go live.</t>
         </is>
       </c>
       <c r="G4" s="14" t="inlineStr">
@@ -2225,7 +2222,7 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr"/>

</xml_diff>